<commit_message>
docs(sop): add GM, Fashion, and LP & Maintenance audit checklists
Three new sheets added to SOP_Audit_Checklists.xlsx:
- GM Audit Tool (100 marks, 5 sections, 22 criteria)
- Fashion Audit Tool (100 marks, 4 sections, 24 criteria)
- LP & Maintenance SOP Audit (96 marks, 7 sections, 41 criteria)

All three are new tools not previously in the workbook.
Existing Cash and FMCG sheets are unchanged.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SOP_Audit_Checklists.xlsx
+++ b/docs/SOP_Audit_Checklists.xlsx
@@ -1,14 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Audit Tool" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FMCG Audit Tool" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cash Audit Tool" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="FMCG Audit Tool" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="GM Audit Tool" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Fashion Audit Tool" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="LP &amp; Maintenance Audit" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,8 +43,35 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0000338D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -83,8 +113,33 @@
         <fgColor rgb="00FFD966"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000338D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000061A6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C7D9F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEAF8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -106,11 +161,69 @@
         <color rgb="00BBBBBB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -146,6 +259,38 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -569,6 +714,11 @@
           <t>Section A: Back Office Management   |   Total Marks: 16</t>
         </is>
       </c>
+      <c r="B3" s="13" t="n"/>
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="14" t="n"/>
     </row>
     <row r="4" ht="77" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -790,6 +940,11 @@
           <t>Section B: Front End Management   |   Total Marks: 21</t>
         </is>
       </c>
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="14" t="n"/>
     </row>
     <row r="13" ht="99" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
@@ -932,6 +1087,11 @@
           <t>Section C: People Management   |   Total Marks: 20</t>
         </is>
       </c>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="14" t="n"/>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
@@ -1043,6 +1203,11 @@
           <t>Section D: Customer Relationship Management   |   Total Marks: 5</t>
         </is>
       </c>
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="13" t="n"/>
+      <c r="D23" s="13" t="n"/>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="14" t="n"/>
     </row>
     <row r="24" ht="60" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -1076,6 +1241,11 @@
           <t>Section E: Merchandise Management   |   Total Marks: 15</t>
         </is>
       </c>
+      <c r="B25" s="13" t="n"/>
+      <c r="C25" s="13" t="n"/>
+      <c r="D25" s="13" t="n"/>
+      <c r="E25" s="13" t="n"/>
+      <c r="F25" s="14" t="n"/>
     </row>
     <row r="26" ht="60" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
@@ -1230,6 +1400,11 @@
           <t>Section A: Bay Management Audit   |   Total Marks: 32</t>
         </is>
       </c>
+      <c r="B3" s="13" t="n"/>
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="14" t="n"/>
     </row>
     <row r="4" ht="120" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -1440,6 +1615,11 @@
           <t>Section B: Pricing   |   Total Marks: 12</t>
         </is>
       </c>
+      <c r="B10" s="13" t="n"/>
+      <c r="C10" s="13" t="n"/>
+      <c r="D10" s="13" t="n"/>
+      <c r="E10" s="13" t="n"/>
+      <c r="F10" s="14" t="n"/>
     </row>
     <row r="11" ht="120" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
@@ -1549,6 +1729,11 @@
           <t>Section C: People Management Audit   |   Total Marks: 24</t>
         </is>
       </c>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="14" t="n"/>
     </row>
     <row r="15" ht="111" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
@@ -1742,6 +1927,11 @@
           <t>Section D: Merchandize Management Audit   |   Total Marks: 24</t>
         </is>
       </c>
+      <c r="B21" s="13" t="n"/>
+      <c r="C21" s="13" t="n"/>
+      <c r="D21" s="13" t="n"/>
+      <c r="E21" s="13" t="n"/>
+      <c r="F21" s="14" t="n"/>
     </row>
     <row r="22" ht="114" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -1949,6 +2139,11 @@
           <t>Section E: Category Management   |   Total Marks: 8</t>
         </is>
       </c>
+      <c r="B28" s="13" t="n"/>
+      <c r="C28" s="13" t="n"/>
+      <c r="D28" s="13" t="n"/>
+      <c r="E28" s="13" t="n"/>
+      <c r="F28" s="14" t="n"/>
     </row>
     <row r="29" ht="120" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
@@ -2022,4 +2217,3253 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>GM Audit Tool - SOP Checklist   |   Audit Date: 6/11/2021   |   Total Marks: 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Marks</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>Maximum (Best in Class)</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>Average (50% of Max)</t>
+        </is>
+      </c>
+      <c r="E2" s="16" t="inlineStr">
+        <is>
+          <t>Minimum (Zero)</t>
+        </is>
+      </c>
+      <c r="F2" s="16" t="inlineStr">
+        <is>
+          <t>Actual Score</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Section A: Bay Management Audit   |   Total Marks: 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Planogram Adherence</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>6 Bays checked at random:
+- No missing SELs, perfectly left aligned
+- Stock spread as per planogram guidelines
+- Planno file available in aisle itself
+- NPI added only in right side of relevant shelf
+- No damaged stock found</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>6 Bays checked at random:
+- Less than 4 missing SELs; left alignment improvable
+- Some gaps in shelves; planno file available in aisle</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>6 Bays checked at random:
+- More than 4 missing SELs; alignment quite bad
+- Planno file not in aisle; NPI added randomly
+- Damaged stock found</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="n"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>Visibility Management</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>- All endcaps and sidecaps merchandised as per Visibility plan
+- Visibility file checked weekly and cross-checked by SBM
+- VM rules regarding signages &amp; dropdown fully followed</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>- Endcaps merchandised per visibility file but stock-out exceptions not managed
+- Visibility file maintained but not checked weekly</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>- Visibility file not well managed
+- Impulse bays badly managed; VM rules flouted</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="n"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Shelves and Merchandize are neat without any dust</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>- All shelves fully dusted and cleaned
+- No damage or soiled packs on shelves
+- Gondola ends and top shelves dust-free
+- Floor under shelves swept and clean</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>- Most shelves dusted; minor dust at top shelves
+- 1-2 damaged packs visible; floor mostly clean</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>- Visible dust on shelves and gondola tops
+- Multiple damaged or soiled packs on display</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="n"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>Merchandise on Floor Ready for Sale</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>- All merchandise on floor is in perfect sellable condition
+- Correct MRP sticker on each item; no missing tags
+- No expired or damaged goods on floor
+- Fill level &gt; 80% across all bays</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>- Majority of merchandise sellable; &lt; 3 items without proper MRP
+- Fill level 60-80%; minor expired stock in one bay</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>- Several items not sale-ready (missing MRP, damaged, expired)
+- Fill level &lt; 60%; expired stock on shelf</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="n"/>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Floor Management</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>- Aisles completely clear; no boxes/pallets on floor
+- Signage and directional flow correct
+- No empty display spaces</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>- Minor clutter in 1-2 aisles; signage largely correct
+- 1-2 empty display spaces</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>- Multiple aisles obstructed; boxes/pallets blocking flow
+- Significant empty display spaces; signage missing</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>Cleanliness &amp; Hygiene</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>- Store floor spotless; no spillages or debris
+- Washrooms clean and stocked
+- Garbage bins emptied regularly; no odour</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>- Floor mostly clean; minor debris in 1-2 aisles
+- Washrooms acceptable but some consumables missing</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>- Visible spillages or debris on floor
+- Washrooms dirty or unstocked
+- Garbage overflowing; noticeable odour</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Section B: Pricing   |   Total Marks: 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>IT and DH Price Change Coordination and SEL Implementation</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>- 100% price changes implemented on system the same day
+- All SELs updated within SLA; no price mismatch
+- Coordination log between IT and DH maintained</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>- &gt; 90% price changes implemented; &lt; 5 SEL mismatches
+- Minor delays noted</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>- &lt; 90% price changes updated; &gt; 5 SEL mismatches
+- No coordination log maintained</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="n"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t>Visibility Price Signages</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>- All promo price signages correctly displayed
+- No outdated or incorrect signage visible
+- All A4/A6 boards in place with correct content</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>- Most signages correct; 1-2 incorrect or outdated
+- Promo boards mostly in place</t>
+        </is>
+      </c>
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>- Multiple incorrect or outdated signages
+- Promo boards missing or displaying wrong info</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="n"/>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Live More Day / Buying Cycle Price Change Implementation (N/A)</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>- All Live More Day price changes implemented on time
+- Zero missed price changes during the cycle</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>- Most price changes implemented; minor delays in 1-2 categories</t>
+        </is>
+      </c>
+      <c r="E13" s="20" t="inlineStr">
+        <is>
+          <t>- Price changes delayed or missed for multiple categories</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Section C: People Management Audit   |   Total Marks: 24</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Duty Roster</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>- Roster prepared 7 days in advance and displayed
+- 100% adherence to roster; all shifts covered
+- Leave plan approved and documented</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>- Roster prepared 3-5 days in advance; 80-90% adherence
+- 1-2 uncovered shifts; most leaves documented</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>- Roster prepared &lt; 3 days in advance or not displayed
+- &lt; 80% adherence; multiple uncovered shifts</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="n"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>DILO (Day in the Life Of)</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>- Manager DILO completed for all team members this week
+- DILO observations documented with action points
+- Previous DILO actions verified as closed</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>- DILO completed for &gt; 50% of team; observations documented
+- Some actions from previous DILO still open</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>- DILO not done or done for &lt; 50% of team
+- No documentation of observations or action points</t>
+        </is>
+      </c>
+      <c r="F16" s="21" t="n"/>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Grooming Standard</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>- 100% staff in proper uniform with name badge
+- Hair neatly groomed; shoes polished
+- No casual wear, jewellery, or mobile phones visible on floor</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>- &gt; 90% staff in proper uniform; 1-2 without name badge
+- Minor grooming lapses noted</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>- &lt; 90% staff in uniform; multiple grooming violations
+- Staff without name badges and with casual wear</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="n"/>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>Promoters</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="24" t="inlineStr">
+        <is>
+          <t>- All promoters in brand uniform and at designated locations
+- Promoter attendance logged and on time
+- Promoters actively engaging customers</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="inlineStr">
+        <is>
+          <t>- Most promoters in uniform and at location; 1 absent
+- Engagement levels moderate</t>
+        </is>
+      </c>
+      <c r="E18" s="24" t="inlineStr">
+        <is>
+          <t>- Promoters not in uniform, absent, or not at designated locations
+- No engagement with customers</t>
+        </is>
+      </c>
+      <c r="F18" s="21" t="n"/>
+    </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>Staff Knowledge</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>- Staff can accurately explain product features, pricing &amp; promotions
+- 3 random staff tested -- all score &gt; 80%
+- Knowledge boards/materials available and updated</t>
+        </is>
+      </c>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>- Staff have basic knowledge; 1-2 gaps in promo awareness
+- 3 random staff -- average score 50-80%</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="inlineStr">
+        <is>
+          <t>- Staff unable to answer basic product or promo queries
+- 3 random staff -- average score &lt; 50%</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Section D: Merchandize Management Audit   |   Total Marks: 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Pick List</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>- Pick list generated daily and actioned within TAT
+- 100% of picks verified and signed off
+- No pending picks older than 1 day</t>
+        </is>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>- Pick list generated; 80-90% actioned within TAT
+- 1-2 picks older than 1 day</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>- Pick list not generated daily or actioned late
+- Multiple unverified picks; picks older than 2+ days</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="n"/>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>Fill Rates</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>- On-shelf fill rate &gt; 95% across all categories
+- Out-of-stock replenished within 2 hours
+- Fill rate tracker maintained and reviewed daily</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>- Fill rate 85-95%; most OOS replenished within 4 hours</t>
+        </is>
+      </c>
+      <c r="E22" s="24" t="inlineStr">
+        <is>
+          <t>- Fill rate &lt; 85%; OOS not tracked or replenished promptly</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="n"/>
+    </row>
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Shrinkage Management</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" s="20" t="inlineStr">
+        <is>
+          <t>- Shrinkage &lt; budget; all variances investigated
+- Tagging compliance 100%; CCTV monitored
+- Shrinkage hotspots identified and actioned</t>
+        </is>
+      </c>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>- Shrinkage within 10% of budget; most variances documented
+- Tagging compliance &gt; 90%</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="inlineStr">
+        <is>
+          <t>- Shrinkage &gt; budget with no investigation
+- Tagging compliance &lt; 90%</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="n"/>
+    </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>Clearance &amp; Liquidation</t>
+        </is>
+      </c>
+      <c r="B24" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" s="24" t="inlineStr">
+        <is>
+          <t>- Clearance merchandise in designated area with proper signage
+- Liquidation plan reviewed weekly; stock moving as planned
+- Zero expired clearance stock on floor</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>- Clearance area mostly organized; minor signage issues
+- Some slow-moving stock without plan</t>
+        </is>
+      </c>
+      <c r="E24" s="24" t="inlineStr">
+        <is>
+          <t>- Clearance merchandise scattered or without proper signage
+- No active liquidation plan; expired clearance stock present</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="n"/>
+    </row>
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>WBC (N/A)</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>- WBC count done as per schedule; all discrepancies resolved
+- WBC records maintained and signed off by manager</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>- WBC count done; minor discrepancies not fully resolved</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>- WBC count not done on schedule; discrepancies unresolved</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="n"/>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>Backroom / Remote WH Management</t>
+        </is>
+      </c>
+      <c r="B26" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="C26" s="24" t="inlineStr">
+        <is>
+          <t>- Backroom immaculate: all stock location-labelled and organized
+- FIFO followed strictly; no blocked fire exits
+- Remote WH stock reconciled weekly</t>
+        </is>
+      </c>
+      <c r="D26" s="24" t="inlineStr">
+        <is>
+          <t>- Backroom mostly organized; minor labelling gaps
+- FIFO mostly followed; one minor fire exit concern</t>
+        </is>
+      </c>
+      <c r="E26" s="24" t="inlineStr">
+        <is>
+          <t>- Backroom disorganized; stock blocking pathways
+- FIFO not followed; fire exit blocked</t>
+        </is>
+      </c>
+      <c r="F26" s="21" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Section E: Category Management   |   Total Marks: 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Benchmarking</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>- Competitor benchmarking done this week with documented insights
+- Benchmarking report shared with category team
+- Action plan created based on benchmarking findings</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>- Benchmarking done this month; insights partially documented
+- Report shared but action plan incomplete</t>
+        </is>
+      </c>
+      <c r="E28" s="20" t="inlineStr">
+        <is>
+          <t>- Benchmarking not done in last 2 weeks
+- No documentation or action plan</t>
+        </is>
+      </c>
+      <c r="F28" s="21" t="n"/>
+    </row>
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>RTV (Return to Vendor)</t>
+        </is>
+      </c>
+      <c r="B29" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="24" t="inlineStr">
+        <is>
+          <t>- All RTVs raised within SLA; vendor acknowledgements received
+- RTV tracker updated and reviewed weekly</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>- Most RTVs raised on time; 1-2 delayed
+- Tracker mostly updated</t>
+        </is>
+      </c>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>- RTVs not raised on time; vendor acknowledgements missing
+- No RTV tracker maintained</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="n"/>
+    </row>
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>Demo Management (N/A)</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>- Demo schedule displayed and strictly followed
+- Demo stations clean and fully stocked
+- Customer engagement during demo excellent; sales conversion tracked</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>- Demo schedule mostly followed; 1 station not stocked
+- Moderate customer engagement</t>
+        </is>
+      </c>
+      <c r="E30" s="20" t="inlineStr">
+        <is>
+          <t>- Demo schedule not followed or not displayed
+- Demo stations dirty or empty; no customer engagement</t>
+        </is>
+      </c>
+      <c r="F30" s="21" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A20:F20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Fashion Audit Tool - SOP Checklist   |   Audit Date: 6/18/2021   |   Total Marks: 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Marks</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>Maximum (Best in Class)</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>Average (50% of Max)</t>
+        </is>
+      </c>
+      <c r="E2" s="16" t="inlineStr">
+        <is>
+          <t>Minimum (Zero)</t>
+        </is>
+      </c>
+      <c r="F2" s="16" t="inlineStr">
+        <is>
+          <t>Actual Score</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Section A: Floor Management Audit   |   Total Marks: 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Shelves and Merchandize are neat without any dust</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>- All shelves, folded stacks, and hanging rails dust-free
+- No damaged or soiled garments on display
+- Fixtures wiped down daily</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>- Most shelves clean; minor dust on top shelves
+- 1-2 damaged garments visible</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>- Visible dust on shelves and fixtures
+- Multiple damaged or soiled garments on display</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="n"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>Cleanliness &amp; Hygiene</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>- Floor spotless; no debris, threads, or hangers on floor
+- Trial rooms clean and deodorized after each use
+- Garbage bins emptied regularly</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>- Floor mostly clean; minor debris near fitting rooms
+- Trial rooms clean but not consistently deodorized</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>- Visible debris/threads on floor
+- Trial rooms dirty or with strong odour
+- Garbage overflowing</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="n"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Racking Capacity Tracker</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>- Racking capacity tracker updated daily
+- No fixture overloaded beyond 85% capacity
+- Capacity trends used to plan replenishment</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>- Tracker updated; 1-2 fixtures at &gt; 85% capacity
+- Replenishment plan partially linked to tracker</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>- Tracker not updated regularly
+- Multiple fixtures overloaded; no replenishment plan</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="n"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>Innerwear Size Sets</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>- All innerwear size runs complete (S to XXL / 38-44)
+- Peg hooks fully stocked; no empty hooks
+- Size labels clearly visible on all fixtures</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>- &gt; 80% size runs complete; minor gaps in 1-2 sizes
+- Most peg hooks stocked; 1-2 empty hooks</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>- &lt; 80% size runs complete; multiple size gaps
+- Peg hooks with visible empty spaces; size labels missing</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="n"/>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Folding</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>- All folded merchandise uniformly folded to standard
+- Face-out and fold-out displays perfectly aligned
+- Folding re-done after every customer interaction</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>- Most merchandise folded; minor inconsistency in 1-2 fixtures
+- Face-out displays mostly aligned</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>- Folding inconsistent or not to standard
+- Multiple fixtures with unfolded/thrown merchandise</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>Merchandise Arrangement</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>- Merchandise arranged by colour, size, and category as per VM guidelines
+- Adjacencies followed; power walls executed correctly
+- Price points clearly zoned</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>- Arrangement mostly correct; minor deviations in 1-2 zones
+- Power wall concept partially executed</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>- No clear merchandise arrangement strategy
+- Colours and sizes mixed; VM guidelines not followed</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="n"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Replenishment</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>- Replenishment done within 2 hours of stock reaching minimum level
+- All sizes replenished to full; no empty pegs/slots
+- Replenishment log maintained and signed off</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>- Replenishment done within 4 hours; most sizes refilled
+- 1-2 empty pegs; log maintained</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>- Replenishment delayed &gt; 4 hours; multiple empty pegs
+- No replenishment log</t>
+        </is>
+      </c>
+      <c r="F10" s="21" t="n"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>Mannequin Displays, Hot Spots, Focal Point &amp; High Point (N/A)</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>- All mannequins dressed as per current VM directive
+- Hot spots and focal points highlighted with correct signage
+- High point displays changed weekly</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>- Most mannequins dressed correctly; 1 mannequin not per directive
+- Hot spots mostly executed; minor signage gaps</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>- Mannequins not dressed per VM directive or undressed
+- Hot spots and focal points not identified or executed</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="n"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Ironing</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>- 100% of merchandise on display is wrinkle-free
+- Ironing station operational and staffed
+- New receipts ironed before going on floor</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>- &gt; 90% merchandise wrinkle-free; 1-2 items need ironing
+- Ironing station operational but not always staffed</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>- Visible wrinkled merchandise on display
+- Ironing station not operational or unstaffed</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="n"/>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>Trials</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>- Trial room queue managed; waiting time &lt; 5 mins
+- Maximum items per trial enforced; tagging in place
+- Trial rooms inspected and reset every 30 mins</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>- Trial room queue managed; occasional &gt; 5 min wait
+- Most trial rooms reset; 1 inspection gap per hour</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="inlineStr">
+        <is>
+          <t>- Trial room queue unmanaged; long waits
+- Trial rooms not reset; tagging not enforced</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Section B: Pricing   |   Total Marks: 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>IT and DH Price Change Coordination and SEL Implementation</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>- 100% price changes implemented same day; SELs updated within SLA
+- No price mismatch between system and SEL</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>- &gt; 90% price changes implemented; &lt; 3 SEL mismatches</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>- &lt; 90% price changes updated; multiple SEL mismatches</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="n"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>Visibility Price Signages</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>- All promo price signages correct and displayed at right locations
+- Outdated signage removed immediately after promo end</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>- Most signages correct; 1 outdated or incorrectly placed signage</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>- Multiple incorrect or outdated signages visible</t>
+        </is>
+      </c>
+      <c r="F16" s="21" t="n"/>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Live More Day / Buying Cycle Price Change Implementation (N/A)</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>- All buying cycle price changes actioned same day
+- Zero missed price changes during cycle</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>- Most price changes implemented; minor delays</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>- Price changes delayed or missed for multiple categories</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="n"/>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>WBC Count</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="24" t="inlineStr">
+        <is>
+          <t>- WBC count completed as per schedule with zero discrepancy
+- Records signed off by duty manager</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="inlineStr">
+        <is>
+          <t>- WBC count done; minor discrepancy documented</t>
+        </is>
+      </c>
+      <c r="E18" s="24" t="inlineStr">
+        <is>
+          <t>- WBC count not done on schedule; discrepancy unresolved</t>
+        </is>
+      </c>
+      <c r="F18" s="21" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Section C: People Management Audit   |   Total Marks: 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Selling Skills</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>- Staff approach all customers within 30 seconds of entry
+- AIDAR selling technique followed; add-on selling observed
+- Staff demonstrate product knowledge during interaction</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>- Staff approach most customers; some delays in greeting
+- Basic selling technique used; add-on selling inconsistent</t>
+        </is>
+      </c>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>- Staff do not approach customers or greet poorly
+- No selling technique; no add-on selling observed</t>
+        </is>
+      </c>
+      <c r="F20" s="21" t="n"/>
+    </row>
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>Work With CSA / Role Play</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>- Formal work-with session done with each CSA this week
+- Role play conducted for at least 2 scenarios
+- Feedback given and improvement plan documented</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>- Work-with done for &gt; 50% of CSAs; 1 role play completed
+- Basic feedback given</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>- Work-with sessions not done or &lt; 50% CSAs covered
+- No role play conducted</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="n"/>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>DILO (Day in the Life Of)</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>- Manager DILO completed for all team members this week
+- DILO observations documented with action points
+- Previous DILO actions verified as closed</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>- DILO completed for &gt; 50% of team; observations documented
+- Some previous actions still open</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>- DILO not done or done for &lt; 50% of team
+- No documentation or actions</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="n"/>
+    </row>
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>Grooming Standard</t>
+        </is>
+      </c>
+      <c r="B23" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" s="24" t="inlineStr">
+        <is>
+          <t>- 100% staff in proper uniform with name badge
+- Hair neatly groomed; no casual wear or jewellery
+- Fragrance and footwear per standard</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>- &gt; 90% staff in proper uniform; 1-2 minor grooming lapses</t>
+        </is>
+      </c>
+      <c r="E23" s="24" t="inlineStr">
+        <is>
+          <t>- &lt; 90% in uniform; multiple grooming violations</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="n"/>
+    </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Promoters</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>- All brand promoters in uniform and at designated location
+- Attendance logged; promoters actively engaging customers</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>- Most promoters in uniform; 1 absent or off-location
+- Engagement moderate</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>- Promoters not in uniform, absent, or not engaging customers</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Section D: Merchandize Management Audit   |   Total Marks: 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>Quality &amp; Customer Returns Management</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>- Returns processed within 24 hrs per policy
+- Returns log maintained; defect analysis done weekly
+- Returned merchandise re-checked before going back to floor</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>- Returns processed within 48 hrs; log maintained
+- Defect analysis done monthly</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>- Returns processed &gt; 48 hrs or without policy adherence
+- No returns log or defect analysis</t>
+        </is>
+      </c>
+      <c r="F26" s="21" t="n"/>
+    </row>
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>Customer Conversion Optimization</t>
+        </is>
+      </c>
+      <c r="B27" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" s="24" t="inlineStr">
+        <is>
+          <t>- Conversion rate tracked daily; footfall vs. billing ratio reviewed
+- Actions taken for conversion dips; incentive plan active
+- Conversion &gt; store target</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="inlineStr">
+        <is>
+          <t>- Conversion tracked; actions taken but not consistently
+- Conversion within 5% of target</t>
+        </is>
+      </c>
+      <c r="E27" s="24" t="inlineStr">
+        <is>
+          <t>- Conversion rate not tracked; no actions for dips
+- Conversion &gt; 10% below target</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="n"/>
+    </row>
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Shrinkage Management</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>- Shrinkage &lt; budget; all variances investigated and closed
+- Soft tagging on 100% high-value merchandise
+- CCTV monitored at hotspots</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>- Shrinkage within 10% of budget; most variances documented
+- Tagging compliance &gt; 90%</t>
+        </is>
+      </c>
+      <c r="E28" s="20" t="inlineStr">
+        <is>
+          <t>- Shrinkage &gt; budget; no investigation
+- Tagging compliance &lt; 90%</t>
+        </is>
+      </c>
+      <c r="F28" s="21" t="n"/>
+    </row>
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>Alteration Management</t>
+        </is>
+      </c>
+      <c r="B29" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="24" t="inlineStr">
+        <is>
+          <t>- Alteration TAT &lt; 48 hrs; customer informed on time
+- Alteration log maintained; 100% customer sign-off on delivery
+- Zero re-dos due to quality issues</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>- Alteration TAT &lt; 72 hrs; most customers informed
+- Log maintained; 1-2 re-dos</t>
+        </is>
+      </c>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>- Alteration TAT &gt; 72 hrs; customers not informed
+- No alteration log; multiple re-dos</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="n"/>
+    </row>
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>Clearance &amp; Liquidation</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>- Clearance zone clean, organized, and clearly signposted
+- Liquidation plan reviewed weekly; stock moving on target
+- Zero expired/past-season stock on main floor</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>- Clearance zone mostly organized; minor signage issues
+- Liquidation plan reviewed monthly</t>
+        </is>
+      </c>
+      <c r="E30" s="20" t="inlineStr">
+        <is>
+          <t>- Clearance zone scattered or without proper signage
+- No active liquidation plan</t>
+        </is>
+      </c>
+      <c r="F30" s="21" t="n"/>
+    </row>
+    <row r="31" ht="60" customHeight="1">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>Backroom Management</t>
+        </is>
+      </c>
+      <c r="B31" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>- Backroom fully organized; all stock location-labelled
+- FIFO followed; fire exits clear
+- Stock reconciled with system weekly</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="inlineStr">
+        <is>
+          <t>- Backroom mostly organized; minor labelling gaps
+- FIFO mostly followed</t>
+        </is>
+      </c>
+      <c r="E31" s="24" t="inlineStr">
+        <is>
+          <t>- Backroom disorganized; stock blocking pathways
+- FIFO not followed or fire exit obstructed</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A25:F25"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>LP &amp; Maintenance SOP Audit - SOP Checklist   |   Audit Date: 30th June 2021   |   Total Marks: 96</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Marks</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>Maximum (Best in Class)</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>Average (50% of Max)</t>
+        </is>
+      </c>
+      <c r="E2" s="16" t="inlineStr">
+        <is>
+          <t>Minimum (Zero)</t>
+        </is>
+      </c>
+      <c r="F2" s="16" t="inlineStr">
+        <is>
+          <t>Actual Score</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Section A: Back End Management   |   Total Marks: 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Trolley Cleaning</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>- All trolleys cleaned and sanitised daily
+- Cleaning schedule displayed and signed off
+- Defective trolleys removed from service immediately</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>- &gt; 80% trolleys cleaned; cleaning schedule maintained
+- 1-2 defective trolleys still in service</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>- &lt; 80% trolleys cleaned; no cleaning schedule
+- Multiple defective trolleys in service</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="n"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>Trolley Retrieval &amp; Parking Bays</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>- Trolleys retrieved every 30 mins from parking areas
+- Parking bays clearly marked and unobstructed
+- Trolley count reconciled at start and end of day</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>- Trolleys retrieved every 45-60 mins; most bays marked
+- Count reconciled daily</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>- Trolleys not retrieved regularly; parking bays obstructed
+- No trolley count reconciliation</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="n"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Parking Management - Mall / Stand-alone Store (N/A)</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>- Clear parking zones marked for customers and staff
+- Security managing traffic flow at peak times
+- No unauthorized vehicles in customer zones</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>- Parking zones marked; minor unauthorized vehicle issue</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>- Parking zones not clearly marked; unauthorized vehicles in customer zones</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="n"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>Crowd Control and Management</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>- Crowd control plan in place for peak hours and events
+- Queue management at billing and entry/exit
+- Staff trained in crowd management procedures</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>- Crowd control plan exists; 1-2 gaps in execution at peak
+- Queue management mostly in place</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>- No crowd control plan; queues unmanaged
+- Staff not trained in crowd management</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="n"/>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Back Store Management</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>- Back store immaculate; all areas labelled and organised
+- No clutter or unauthorized storage
+- Back store access controlled and logged</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>- Back store mostly organised; minor labelling gaps
+- 1 area of unauthorized storage noted</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>- Back store disorganized; items blocking pathways
+- No access control or log maintained</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>Transportation &amp; Man Management</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>- All transport (receiving/dispatch) scheduled and on time
+- Labour deployment plan available for all transport activities
+- No unauthorized movement of goods</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>- Transport mostly on schedule; 1 delay noted
+- Labour deployment plan available but partially followed</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>- Transport unscheduled; significant delays
+- No labour deployment plan; unauthorized movements</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="n"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Pest Control</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>- Pest control contract active; last treatment within 30 days
+- Pest control register maintained and signed
+- No evidence of pest activity on floor or in back store</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>- Pest control done; register maintained but 1 gap in sign-off
+- Minor evidence of pest activity addressed</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>- Pest control overdue &gt; 30 days; register not maintained
+- Active pest activity visible</t>
+        </is>
+      </c>
+      <c r="F10" s="21" t="n"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>External Warehouse / Remote (N/A)</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>- External WH organized and reconciled weekly
+- Access log maintained; security in place</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>- External WH mostly organized; reconciliation done monthly</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>- External WH disorganized; no reconciliation or security</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="n"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Liasoning</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>- All statutory liaising (municipality, mall authority, fire dept.) up to date
+- Liaison contact list available and current
+- All pending matters followed up within 48 hrs</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>- Most liaising up to date; 1 pending matter &gt; 48 hrs
+- Contact list available but not fully current</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>- Multiple statutory liaising issues overdue
+- No contact list; pending matters not followed up</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Section B: Safety Management   |   Total Marks: 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>EHS Audit Score &amp; NC Closure</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>- Latest EHS audit score &gt; 90%; all NCs closed within SLA
+- NC closure tracker updated and signed off by manager</t>
+        </is>
+      </c>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>- EHS score 75-90%; &gt; 80% NCs closed within SLA</t>
+        </is>
+      </c>
+      <c r="E14" s="20" t="inlineStr">
+        <is>
+          <t>- EHS score &lt; 75%; &gt; 20% NCs overdue
+- Tracker not maintained</t>
+        </is>
+      </c>
+      <c r="F14" s="21" t="n"/>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>OHSAS Audit Score</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="24" t="inlineStr">
+        <is>
+          <t>- OHSAS audit score &gt; 90%; certificate current
+- All OHSAS requirements documented and complied with</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>- OHSAS score 75-90%; certificate current; minor compliance gaps</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>- OHSAS score &lt; 75% or certificate expired</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="n"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Stretcher Availability</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>- Stretcher in designated location, accessible, and fully equipped
+- Staff trained in stretcher use
+- Stretcher log signed weekly</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>- Stretcher available but 1 accessory missing
+- Most staff trained; log signed monthly</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>- Stretcher missing, inaccessible, or poorly equipped
+- Staff not trained; no log</t>
+        </is>
+      </c>
+      <c r="F16" s="21" t="n"/>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>Fire Extinguishers</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>- All fire extinguishers charged, inspected monthly, and accessible
+- Inspection tags current on all units
+- No extinguisher obstructed</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>- &gt; 90% extinguishers charged and inspected; 1 minor obstruction
+- Most tags current</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>- &lt; 90% extinguishers charged or inspected
+- Multiple extinguishers obstructed or tags expired</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="n"/>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>AC / DG / Electrical Rooms</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>- All AC, DG, and electrical rooms locked, clean, and access-controlled
+- Maintenance log updated; no unauthorized access
+- SOP signage displayed in all rooms</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>- Rooms mostly secured; 1 minor access or cleanliness issue</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>- Rooms unlocked, dirty, or with unauthorized access
+- Maintenance log not maintained</t>
+        </is>
+      </c>
+      <c r="F18" s="21" t="n"/>
+    </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>Fire Exits</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="24" t="inlineStr">
+        <is>
+          <t>- All fire exits unobstructed, clearly marked, and illuminated
+- Exit routes checked daily; no storage near exits
+- Fire exit drill conducted in last 6 months</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="inlineStr">
+        <is>
+          <t>- Fire exits unobstructed; 1 signage or lighting issue
+- Routes checked weekly; drill done in last 12 months</t>
+        </is>
+      </c>
+      <c r="E19" s="24" t="inlineStr">
+        <is>
+          <t>- Fire exits obstructed or unmarked
+- No regular checks; no drill in last 12 months</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="n"/>
+    </row>
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Reporting of Accident &amp; Incident</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>- All accidents/incidents reported within 1 hr using standard form
+- Incident register maintained and up to date
+- Root cause analysis done for all incidents</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>- Most incidents reported within 24 hrs; register maintained
+- RCA done for major incidents only</t>
+        </is>
+      </c>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>- Incidents not reported or delayed &gt; 24 hrs
+- No incident register or RCA</t>
+        </is>
+      </c>
+      <c r="F20" s="21" t="n"/>
+    </row>
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>FSMS (Food Safety Management System)</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>- FSMS checklist completed daily and signed off
+- All FSMS NCs closed within 24 hrs
+- FSMS training completed for all relevant staff</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>- FSMS checklist completed on most days; NCs closed within 48 hrs</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>- FSMS checklist not completed regularly
+- NCs not tracked or training not conducted</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Section C: Housekeeping Management   |   Total Marks: 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Floor Cleanliness</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" s="20" t="inlineStr">
+        <is>
+          <t>- All floor areas swept and mopped every 2 hours
+- No spillages, stains, or debris on floor
+- Cleaning schedule signed off every shift</t>
+        </is>
+      </c>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>- Floor cleaned every 4 hours; minor stain or debris visible</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="inlineStr">
+        <is>
+          <t>- Floor not cleaned per schedule; visible stains and debris
+- No cleaning schedule sign-off</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="n"/>
+    </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>Manpower Availability &amp; Training</t>
+        </is>
+      </c>
+      <c r="B24" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="24" t="inlineStr">
+        <is>
+          <t>- 100% housekeeping manpower deployed as per plan
+- All HK staff trained on cleaning standards and chemical handling
+- Training records updated and available</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>- &gt; 90% manpower deployed; training done for &gt; 80% staff</t>
+        </is>
+      </c>
+      <c r="E24" s="24" t="inlineStr">
+        <is>
+          <t>- &lt; 90% manpower deployed; training incomplete
+- No training records</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="n"/>
+    </row>
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Washrooms Cleanliness &amp; Hygiene</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>- Washrooms inspected every 30 mins and signed on board
+- All consumables (soap, tissue, sanitizer) fully stocked
+- No odour; tiles and fixtures spotless</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>- Washrooms inspected hourly; 1 consumable partially low
+- Minor odour or staining noted</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>- Washrooms inspected &lt; once per 2 hrs; consumables empty
+- Strong odour; tiles or fixtures visibly dirty</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="n"/>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>Housekeeping Consumables &amp; Cleaning Machines</t>
+        </is>
+      </c>
+      <c r="B26" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" s="24" t="inlineStr">
+        <is>
+          <t>- Minimum 7-day stock of all HK consumables maintained
+- All cleaning machines operational and serviced
+- Inventory register updated weekly</t>
+        </is>
+      </c>
+      <c r="D26" s="24" t="inlineStr">
+        <is>
+          <t>- 3-7 day stock of consumables; 1 minor machine issue</t>
+        </is>
+      </c>
+      <c r="E26" s="24" t="inlineStr">
+        <is>
+          <t>- &lt; 3 day stock of consumables; machine breakdowns unresolved
+- No inventory register</t>
+        </is>
+      </c>
+      <c r="F26" s="21" t="n"/>
+    </row>
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Housekeeping Uniforms</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="20" t="inlineStr">
+        <is>
+          <t>- 100% HK staff in clean, intact uniform with ID badge
+- Uniform issue register maintained
+- No staff in casual or personal clothing</t>
+        </is>
+      </c>
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>- &gt; 90% HK staff in uniform; 1 staff without badge</t>
+        </is>
+      </c>
+      <c r="E27" s="20" t="inlineStr">
+        <is>
+          <t>- &lt; 90% HK staff in uniform; multiple without badges
+- No uniform register</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="n"/>
+    </row>
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
+          <t>Deep / Master Cleaning Schedule</t>
+        </is>
+      </c>
+      <c r="B28" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" s="24" t="inlineStr">
+        <is>
+          <t>- Deep cleaning schedule displayed and followed monthly
+- All deep cleaning sign-offs available
+- Deep cleaning covers all zones including ceiling and HVAC</t>
+        </is>
+      </c>
+      <c r="D28" s="24" t="inlineStr">
+        <is>
+          <t>- Deep cleaning done; 1-2 areas not covered or sign-off missing</t>
+        </is>
+      </c>
+      <c r="E28" s="24" t="inlineStr">
+        <is>
+          <t>- No deep cleaning schedule; cleaning not done or undocumented</t>
+        </is>
+      </c>
+      <c r="F28" s="21" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Section D: Security &amp; Shrinkage   |   Total Marks: 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>Security Deployment Plan</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>- Deployment plan posted and followed 100%
+- All positions covered per plan at all times
+- Supervisor checks deployment every 2 hours</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>- Deployment plan posted; 1-2 positions occasionally uncovered</t>
+        </is>
+      </c>
+      <c r="E30" s="20" t="inlineStr">
+        <is>
+          <t>- Deployment plan not posted or not followed
+- Multiple positions uncovered; no supervisor checks</t>
+        </is>
+      </c>
+      <c r="F30" s="21" t="n"/>
+    </row>
+    <row r="31" ht="60" customHeight="1">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>Security Guard Training</t>
+        </is>
+      </c>
+      <c r="B31" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>- All security staff trained on SOP, emergency procedures, and shoplifting detection
+- Training records updated quarterly
+- Mock drills conducted in last 3 months</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="inlineStr">
+        <is>
+          <t>- &gt; 80% staff trained; records updated semi-annually
+- 1 mock drill in last 6 months</t>
+        </is>
+      </c>
+      <c r="E31" s="24" t="inlineStr">
+        <is>
+          <t>- &lt; 80% staff trained; outdated records
+- No mock drills conducted</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="n"/>
+    </row>
+    <row r="32" ht="60" customHeight="1">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>Security Guard Having All Key Contact Numbers</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>- All guards have updated contact list (manager, police, fire, ambulance)
+- Contact list displayed at all guard posts</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="inlineStr">
+        <is>
+          <t>- Guards have contact list; 1-2 numbers outdated
+- List displayed at main post only</t>
+        </is>
+      </c>
+      <c r="E32" s="20" t="inlineStr">
+        <is>
+          <t>- Contact list not available or outdated
+- List not displayed</t>
+        </is>
+      </c>
+      <c r="F32" s="21" t="n"/>
+    </row>
+    <row r="33" ht="60" customHeight="1">
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>Physical Fitness and Age as per Contract</t>
+        </is>
+      </c>
+      <c r="B33" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" s="24" t="inlineStr">
+        <is>
+          <t>- All guards within contractual age (21-45) and physically fit
+- Medical fitness certificate available for all</t>
+        </is>
+      </c>
+      <c r="D33" s="24" t="inlineStr">
+        <is>
+          <t>- &gt; 90% guards within age and fitness standard; 1 minor exception documented</t>
+        </is>
+      </c>
+      <c r="E33" s="24" t="inlineStr">
+        <is>
+          <t>- Multiple guards outside contractual age or below fitness standard
+- No medical certificates</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="n"/>
+    </row>
+    <row r="34" ht="60" customHeight="1">
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>Security Dues Payment</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" s="20" t="inlineStr">
+        <is>
+          <t>- Security vendor payment released on time every month
+- No outstanding dues; payment receipts filed
+- Vendor acknowledgement of receipt on record</t>
+        </is>
+      </c>
+      <c r="D34" s="20" t="inlineStr">
+        <is>
+          <t>- Payment released within 5 days of due date; receipts mostly filed</t>
+        </is>
+      </c>
+      <c r="E34" s="20" t="inlineStr">
+        <is>
+          <t>- Payment delayed &gt; 5 days or outstanding dues not resolved
+- No receipts or vendor acknowledgement</t>
+        </is>
+      </c>
+      <c r="F34" s="21" t="n"/>
+    </row>
+    <row r="35" ht="60" customHeight="1">
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>Security Uniforms</t>
+        </is>
+      </c>
+      <c r="B35" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" s="24" t="inlineStr">
+        <is>
+          <t>- 100% security staff in complete, clean uniform with visible ID
+- Uniform issue and return register maintained
+- No guard in personal clothing</t>
+        </is>
+      </c>
+      <c r="D35" s="24" t="inlineStr">
+        <is>
+          <t>- &gt; 90% in full uniform; 1 guard with minor issue</t>
+        </is>
+      </c>
+      <c r="E35" s="24" t="inlineStr">
+        <is>
+          <t>- &lt; 90% in full uniform; guards without ID
+- No uniform register</t>
+        </is>
+      </c>
+      <c r="F35" s="21" t="n"/>
+    </row>
+    <row r="36" ht="60" customHeight="1">
+      <c r="A36" s="18" t="inlineStr">
+        <is>
+          <t>Tagging of Merchandise (Hard &amp; Soft Tag)</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" s="20" t="inlineStr">
+        <is>
+          <t>- 100% high-value merchandise hard-tagged; soft-tagged per category
+- Tag audit done weekly; no missing tags
+- Deactivation rate tracked at POS</t>
+        </is>
+      </c>
+      <c r="D36" s="20" t="inlineStr">
+        <is>
+          <t>- &gt; 95% merchandise tagged; weekly audit done
+- 1-2 missing tags; deactivation tracked</t>
+        </is>
+      </c>
+      <c r="E36" s="20" t="inlineStr">
+        <is>
+          <t>- &lt; 95% merchandise tagged; tag audit not done
+- Multiple missing tags; no deactivation tracking</t>
+        </is>
+      </c>
+      <c r="F36" s="21" t="n"/>
+    </row>
+    <row r="37" ht="60" customHeight="1">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>Cashier Spot Audit Check</t>
+        </is>
+      </c>
+      <c r="B37" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" s="24" t="inlineStr">
+        <is>
+          <t>- Spot audits on all cashiers completed twice daily
+- Spot audit form signed by supervisor
+- All discrepancies raised and resolved within shift</t>
+        </is>
+      </c>
+      <c r="D37" s="24" t="inlineStr">
+        <is>
+          <t>- Spot audits done once daily; form signed
+- 1-2 discrepancies unresolved at end of shift</t>
+        </is>
+      </c>
+      <c r="E37" s="24" t="inlineStr">
+        <is>
+          <t>- Spot audits not done or done &lt; once daily
+- No form or discrepancy resolution</t>
+        </is>
+      </c>
+      <c r="F37" s="21" t="n"/>
+    </row>
+    <row r="38" ht="60" customHeight="1">
+      <c r="A38" s="18" t="inlineStr">
+        <is>
+          <t>Cash Management (Agency)</t>
+        </is>
+      </c>
+      <c r="B38" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" s="20" t="inlineStr">
+        <is>
+          <t>- Cash pickup by agency on schedule; all documentation complete
+- Cash handled per SOP; no cash left overnight
+- Agency performance reviewed monthly</t>
+        </is>
+      </c>
+      <c r="D38" s="20" t="inlineStr">
+        <is>
+          <t>- Cash pickup mostly on schedule; 1 documentation gap</t>
+        </is>
+      </c>
+      <c r="E38" s="20" t="inlineStr">
+        <is>
+          <t>- Cash pickup delayed or off-schedule; documentation incomplete
+- Cash left overnight or SOP not followed</t>
+        </is>
+      </c>
+      <c r="F38" s="21" t="n"/>
+    </row>
+    <row r="39" ht="60" customHeight="1">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>Customer Exit Gate - Unbilled Tracker</t>
+        </is>
+      </c>
+      <c r="B39" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" s="24" t="inlineStr">
+        <is>
+          <t>- Exit gate unbilled tracker maintained per shift
+- All unbilled merchandise intercepted and resolved
+- Tracker reviewed by manager daily</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>- Tracker maintained; 1-2 unbilled items not fully resolved
+- Reviewed by manager weekly</t>
+        </is>
+      </c>
+      <c r="E39" s="24" t="inlineStr">
+        <is>
+          <t>- Tracker not maintained; unbilled items not tracked
+- No managerial review</t>
+        </is>
+      </c>
+      <c r="F39" s="21" t="n"/>
+    </row>
+    <row r="40" ht="60" customHeight="1">
+      <c r="A40" s="18" t="inlineStr">
+        <is>
+          <t>RGPNRGP (Received Goods / Not Received Goods Process)</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C40" s="20" t="inlineStr">
+        <is>
+          <t>- RGPNRGP process followed 100% at inward; all GRNs raised
+- Discrepancies between PO and delivery documented
+- No pending GRNs older than 24 hrs</t>
+        </is>
+      </c>
+      <c r="D40" s="20" t="inlineStr">
+        <is>
+          <t>- Process followed for &gt; 90% of inwards; 1 pending GRN</t>
+        </is>
+      </c>
+      <c r="E40" s="20" t="inlineStr">
+        <is>
+          <t>- Process not followed consistently; multiple pending GRNs
+- Discrepancies not documented</t>
+        </is>
+      </c>
+      <c r="F40" s="21" t="n"/>
+    </row>
+    <row r="41" ht="60" customHeight="1">
+      <c r="A41" s="22" t="inlineStr">
+        <is>
+          <t>Dump Verification &amp; Proper Disposal</t>
+        </is>
+      </c>
+      <c r="B41" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" s="24" t="inlineStr">
+        <is>
+          <t>- All dump verified against system before disposal
+- Disposal done per SOP with required sign-offs
+- Dump register maintained and reviewed monthly</t>
+        </is>
+      </c>
+      <c r="D41" s="24" t="inlineStr">
+        <is>
+          <t>- Dump verified for &gt; 90% of disposals; register maintained
+- 1 sign-off missing</t>
+        </is>
+      </c>
+      <c r="E41" s="24" t="inlineStr">
+        <is>
+          <t>- Dump not verified before disposal; register not maintained
+- No sign-offs; disposal not per SOP</t>
+        </is>
+      </c>
+      <c r="F41" s="21" t="n"/>
+    </row>
+    <row r="42" ht="60" customHeight="1">
+      <c r="A42" s="18" t="inlineStr">
+        <is>
+          <t>Opening | Closing Process</t>
+        </is>
+      </c>
+      <c r="B42" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" s="20" t="inlineStr">
+        <is>
+          <t>- Opening and closing checklists completed 100% and signed
+- Key holding register maintained; alarm codes documented
+- No exceptions or deviations to process</t>
+        </is>
+      </c>
+      <c r="D42" s="20" t="inlineStr">
+        <is>
+          <t>- Checklists completed; 1 minor item unsigned</t>
+        </is>
+      </c>
+      <c r="E42" s="20" t="inlineStr">
+        <is>
+          <t>- Checklists not completed or unsigned
+- Key holding register not maintained</t>
+        </is>
+      </c>
+      <c r="F42" s="21" t="n"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>Section E: Maintenance Management   |   Total Marks: 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="60" customHeight="1">
+      <c r="A44" s="18" t="inlineStr">
+        <is>
+          <t>Equipment Uptime</t>
+        </is>
+      </c>
+      <c r="B44" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C44" s="20" t="inlineStr">
+        <is>
+          <t>- All equipment uptime &gt; 99%; breakdowns resolved within 4 hrs
+- Uptime tracker updated daily
+- No repeat breakdowns in last 30 days</t>
+        </is>
+      </c>
+      <c r="D44" s="20" t="inlineStr">
+        <is>
+          <t>- Equipment uptime 95-99%; breakdowns resolved within 24 hrs</t>
+        </is>
+      </c>
+      <c r="E44" s="20" t="inlineStr">
+        <is>
+          <t>- Equipment uptime &lt; 95%; breakdowns taking &gt; 24 hrs
+- No uptime tracker</t>
+        </is>
+      </c>
+      <c r="F44" s="21" t="n"/>
+    </row>
+    <row r="45" ht="60" customHeight="1">
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t>P&amp;M Tracker Update</t>
+        </is>
+      </c>
+      <c r="B45" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" s="24" t="inlineStr">
+        <is>
+          <t>- Plant &amp; machinery tracker updated daily with status and next service date
+- All machines with service overdue flagged and actioned</t>
+        </is>
+      </c>
+      <c r="D45" s="24" t="inlineStr">
+        <is>
+          <t>- Tracker updated weekly; 1 machine service slightly overdue</t>
+        </is>
+      </c>
+      <c r="E45" s="24" t="inlineStr">
+        <is>
+          <t>- Tracker not updated; multiple machines with overdue services</t>
+        </is>
+      </c>
+      <c r="F45" s="21" t="n"/>
+    </row>
+    <row r="46" ht="60" customHeight="1">
+      <c r="A46" s="18" t="inlineStr">
+        <is>
+          <t>Preventive Maintenance of All Machines</t>
+        </is>
+      </c>
+      <c r="B46" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C46" s="20" t="inlineStr">
+        <is>
+          <t>- Preventive maintenance done as per schedule for all machines
+- PM completion signed off by engineer and manager
+- Zero machines with overdue PM</t>
+        </is>
+      </c>
+      <c r="D46" s="20" t="inlineStr">
+        <is>
+          <t>- PM done for &gt; 90% of machines; 1 slightly overdue</t>
+        </is>
+      </c>
+      <c r="E46" s="20" t="inlineStr">
+        <is>
+          <t>- PM overdue for &gt; 10% of machines; no sign-offs
+- PM schedule not displayed</t>
+        </is>
+      </c>
+      <c r="F46" s="21" t="n"/>
+    </row>
+    <row r="47" ht="60" customHeight="1">
+      <c r="A47" s="22" t="inlineStr">
+        <is>
+          <t>Filter Cleaning of AC Machines</t>
+        </is>
+      </c>
+      <c r="B47" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" s="24" t="inlineStr">
+        <is>
+          <t>- AC filter cleaning done every 30 days per schedule
+- Filter cleaning log maintained and signed
+- All AC units operational at set temperature</t>
+        </is>
+      </c>
+      <c r="D47" s="24" t="inlineStr">
+        <is>
+          <t>- Filter cleaning done every 45 days; log maintained
+- 1 AC unit at non-standard temperature</t>
+        </is>
+      </c>
+      <c r="E47" s="24" t="inlineStr">
+        <is>
+          <t>- Filter cleaning overdue &gt; 45 days; no log
+- Multiple AC units non-operational or at wrong temperature</t>
+        </is>
+      </c>
+      <c r="F47" s="21" t="n"/>
+    </row>
+    <row r="48" ht="60" customHeight="1">
+      <c r="A48" s="18" t="inlineStr">
+        <is>
+          <t>Cold Room / Island Freezer / DDC Temperatures</t>
+        </is>
+      </c>
+      <c r="B48" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" s="20" t="inlineStr">
+        <is>
+          <t>- All cold room / island freezer / DDC temperatures logged every 2 hours
+- Temperatures within prescribed range 100% of readings
+- Alarms functional and tested monthly</t>
+        </is>
+      </c>
+      <c r="D48" s="20" t="inlineStr">
+        <is>
+          <t>- Temperatures logged every 4 hours; 1-2 readings slightly out of range</t>
+        </is>
+      </c>
+      <c r="E48" s="20" t="inlineStr">
+        <is>
+          <t>- Temperature logging not done or infrequent
+- Multiple out-of-range readings; alarms not tested</t>
+        </is>
+      </c>
+      <c r="F48" s="21" t="n"/>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>Section F: People Management   |   Total Marks: 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="60" customHeight="1">
+      <c r="A50" s="18" t="inlineStr">
+        <is>
+          <t>Duty Roster - Security, HK &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="B50" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" s="20" t="inlineStr">
+        <is>
+          <t>- Roster prepared 7 days in advance for all three functions
+- 100% adherence; all shifts covered
+- Relief arranged for all absentees</t>
+        </is>
+      </c>
+      <c r="D50" s="20" t="inlineStr">
+        <is>
+          <t>- Roster prepared 3-5 days in advance; 80-90% adherence</t>
+        </is>
+      </c>
+      <c r="E50" s="20" t="inlineStr">
+        <is>
+          <t>- Roster &lt; 3 days in advance; &lt; 80% adherence
+- Relief not arranged for absentees</t>
+        </is>
+      </c>
+      <c r="F50" s="21" t="n"/>
+    </row>
+    <row r="51" ht="60" customHeight="1">
+      <c r="A51" s="22" t="inlineStr">
+        <is>
+          <t>Trainings - Security, HK &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="B51" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" s="24" t="inlineStr">
+        <is>
+          <t>- Training calendar displayed and followed
+- All staff trained per plan with attendance records
+- Post-training assessment conducted</t>
+        </is>
+      </c>
+      <c r="D51" s="24" t="inlineStr">
+        <is>
+          <t>- Training mostly per plan; attendance records maintained</t>
+        </is>
+      </c>
+      <c r="E51" s="24" t="inlineStr">
+        <is>
+          <t>- Training calendar not followed; records incomplete
+- No post-training assessments</t>
+        </is>
+      </c>
+      <c r="F51" s="21" t="n"/>
+    </row>
+    <row r="52" ht="60" customHeight="1">
+      <c r="A52" s="18" t="inlineStr">
+        <is>
+          <t>Vendor Management</t>
+        </is>
+      </c>
+      <c r="B52" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="20" t="inlineStr">
+        <is>
+          <t>- All vendor contracts current and reviewed quarterly
+- Vendor performance scorecard maintained
+- Vendor issues escalated and resolved within SLA</t>
+        </is>
+      </c>
+      <c r="D52" s="20" t="inlineStr">
+        <is>
+          <t>- Contracts current; performance scorecard maintained with 1 gap</t>
+        </is>
+      </c>
+      <c r="E52" s="20" t="inlineStr">
+        <is>
+          <t>- Contracts expired or not reviewed; no performance scorecard</t>
+        </is>
+      </c>
+      <c r="F52" s="21" t="n"/>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>Section G: Store Ambience and Customer Experience   |   Total Marks: 13</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="60" customHeight="1">
+      <c r="A54" s="18" t="inlineStr">
+        <is>
+          <t>Wheel Chair - Store or Mall</t>
+        </is>
+      </c>
+      <c r="B54" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" s="20" t="inlineStr">
+        <is>
+          <t>- Minimum 2 wheelchairs available, clean, and in working condition
+- Wheelchair location signposted at entrance
+- Staff trained to assist wheelchair users</t>
+        </is>
+      </c>
+      <c r="D54" s="20" t="inlineStr">
+        <is>
+          <t>- 2 wheelchairs available; 1 minor repair needed
+- Location signposted; staff awareness moderate</t>
+        </is>
+      </c>
+      <c r="E54" s="20" t="inlineStr">
+        <is>
+          <t>- Wheelchairs unavailable, dirty, or non-functional
+- Location not signposted; staff not trained</t>
+        </is>
+      </c>
+      <c r="F54" s="21" t="n"/>
+    </row>
+    <row r="55" ht="60" customHeight="1">
+      <c r="A55" s="22" t="inlineStr">
+        <is>
+          <t>Store Temperature</t>
+        </is>
+      </c>
+      <c r="B55" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" s="24" t="inlineStr">
+        <is>
+          <t>- Store temperature maintained at 22-24 degrees C throughout operating hours
+- Temperature log updated every 2 hours
+- Customer complaints on temperature: zero</t>
+        </is>
+      </c>
+      <c r="D55" s="24" t="inlineStr">
+        <is>
+          <t>- Temperature mostly within range; 1-2 log gaps
+- 1 customer complaint addressed</t>
+        </is>
+      </c>
+      <c r="E55" s="24" t="inlineStr">
+        <is>
+          <t>- Temperature frequently outside range
+- No temperature log; multiple customer complaints</t>
+        </is>
+      </c>
+      <c r="F55" s="21" t="n"/>
+    </row>
+    <row r="56" ht="60" customHeight="1">
+      <c r="A56" s="18" t="inlineStr">
+        <is>
+          <t>Store Music</t>
+        </is>
+      </c>
+      <c r="B56" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" s="20" t="inlineStr">
+        <is>
+          <t>- Approved playlist playing at correct volume (55-65 dB)
+- Music matches store brand and target customer
+- System operational with no interruptions</t>
+        </is>
+      </c>
+      <c r="D56" s="20" t="inlineStr">
+        <is>
+          <t>- Approved playlist playing; volume slightly off or 1 interruption</t>
+        </is>
+      </c>
+      <c r="E56" s="20" t="inlineStr">
+        <is>
+          <t>- Unapproved music; volume too loud/quiet
+- System with frequent interruptions</t>
+        </is>
+      </c>
+      <c r="F56" s="21" t="n"/>
+    </row>
+    <row r="57" ht="60" customHeight="1">
+      <c r="A57" s="22" t="inlineStr">
+        <is>
+          <t>PA System Condition</t>
+        </is>
+      </c>
+      <c r="B57" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" s="24" t="inlineStr">
+        <is>
+          <t>- PA system fully operational; all zones audible
+- Announcements made as per SOP schedule
+- System tested and maintained monthly</t>
+        </is>
+      </c>
+      <c r="D57" s="24" t="inlineStr">
+        <is>
+          <t>- PA system mostly operational; 1 zone with low volume
+- Announcements made but timing inconsistent</t>
+        </is>
+      </c>
+      <c r="E57" s="24" t="inlineStr">
+        <is>
+          <t>- PA system non-operational or with multiple dead zones
+- Announcements not made or poorly executed</t>
+        </is>
+      </c>
+      <c r="F57" s="21" t="n"/>
+    </row>
+    <row r="58" ht="60" customHeight="1">
+      <c r="A58" s="18" t="inlineStr">
+        <is>
+          <t>Loose Assets on Floor &amp; Weekly Count</t>
+        </is>
+      </c>
+      <c r="B58" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" s="20" t="inlineStr">
+        <is>
+          <t>- Weekly loose asset count done and reconciled with register
+- All loose assets tagged and in designated location
+- Zero unaccounted assets in last count</t>
+        </is>
+      </c>
+      <c r="D58" s="20" t="inlineStr">
+        <is>
+          <t>- Weekly count done; 1-2 minor discrepancies resolved</t>
+        </is>
+      </c>
+      <c r="E58" s="20" t="inlineStr">
+        <is>
+          <t>- Count not done weekly; unaccounted assets
+- Assets not tagged or in designated location</t>
+        </is>
+      </c>
+      <c r="F58" s="21" t="n"/>
+    </row>
+    <row r="59" ht="60" customHeight="1">
+      <c r="A59" s="22" t="inlineStr">
+        <is>
+          <t>Scrap &amp; Carton Management</t>
+        </is>
+      </c>
+      <c r="B59" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C59" s="24" t="inlineStr">
+        <is>
+          <t>- Cartons and scrap removed from floor immediately after stocking
+- Scrap disposal done per schedule with documentation
+- No scrap visible in back areas or aisles</t>
+        </is>
+      </c>
+      <c r="D59" s="24" t="inlineStr">
+        <is>
+          <t>- Cartons removed within 2 hours; minor scrap in back area</t>
+        </is>
+      </c>
+      <c r="E59" s="24" t="inlineStr">
+        <is>
+          <t>- Cartons and scrap visible in aisles or back areas
+- No disposal schedule or documentation</t>
+        </is>
+      </c>
+      <c r="F59" s="21" t="n"/>
+    </row>
+    <row r="60" ht="60" customHeight="1">
+      <c r="A60" s="18" t="inlineStr">
+        <is>
+          <t>General Floor Maintenance</t>
+        </is>
+      </c>
+      <c r="B60" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" s="20" t="inlineStr">
+        <is>
+          <t>- Floor surface in perfect condition: no cracks, loose tiles, or uneven surfaces
+- Signage frames and fixtures in good repair
+- Lighting 100% functional in all zones</t>
+        </is>
+      </c>
+      <c r="D60" s="20" t="inlineStr">
+        <is>
+          <t>- Floor surface mostly good; 1 minor crack or loose tile reported
+- 1-2 non-functional lights addressed</t>
+        </is>
+      </c>
+      <c r="E60" s="20" t="inlineStr">
+        <is>
+          <t>- Multiple floor surface issues; fixtures in disrepair
+- Significant lighting failures unaddressed</t>
+        </is>
+      </c>
+      <c r="F60" s="21" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A43:F43"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add GM, Fashion, LP & Maintenance SOP audit tools
- Fixed N/A criteria in 3 new sheets to use numeric marks (4) matching
  FMCG convention; (N/A) in title is the default_na flag, not the cell value
- Added gm/fashion/lp entries to import_sop.py TOOLS dict
- Ran import: GM (5 sec, 23 criteria, 90 marks), Fashion (4 sec, 25 criteria,
  94 marks), LP (7 sec, 51 criteria, 96 marks) published as v1

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SOP_Audit_Checklists.xlsx
+++ b/docs/SOP_Audit_Checklists.xlsx
@@ -139,7 +139,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -219,11 +219,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -293,6 +337,8 @@
     <xf numFmtId="0" fontId="8" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2281,6 +2327,11 @@
           <t>Section A: Bay Management Audit   |   Total Marks: 30</t>
         </is>
       </c>
+      <c r="B3" s="25" t="n"/>
+      <c r="C3" s="25" t="n"/>
+      <c r="D3" s="25" t="n"/>
+      <c r="E3" s="25" t="n"/>
+      <c r="F3" s="26" t="n"/>
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
@@ -2477,6 +2528,11 @@
           <t>Section B: Pricing   |   Total Marks: 8</t>
         </is>
       </c>
+      <c r="B10" s="25" t="n"/>
+      <c r="C10" s="25" t="n"/>
+      <c r="D10" s="25" t="n"/>
+      <c r="E10" s="25" t="n"/>
+      <c r="F10" s="26" t="n"/>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="18" t="inlineStr">
@@ -2544,10 +2600,8 @@
           <t>Live More Day / Buying Cycle Price Change Implementation (N/A)</t>
         </is>
       </c>
-      <c r="B13" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B13" s="19" t="n">
+        <v>4</v>
       </c>
       <c r="C13" s="20" t="inlineStr">
         <is>
@@ -2573,6 +2627,11 @@
           <t>Section C: People Management Audit   |   Total Marks: 24</t>
         </is>
       </c>
+      <c r="B14" s="25" t="n"/>
+      <c r="C14" s="25" t="n"/>
+      <c r="D14" s="25" t="n"/>
+      <c r="E14" s="25" t="n"/>
+      <c r="F14" s="26" t="n"/>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
@@ -2730,6 +2789,11 @@
           <t>Section D: Merchandize Management Audit   |   Total Marks: 20</t>
         </is>
       </c>
+      <c r="B20" s="25" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="26" t="n"/>
     </row>
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="18" t="inlineStr">
@@ -2855,10 +2919,8 @@
           <t>WBC (N/A)</t>
         </is>
       </c>
-      <c r="B25" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B25" s="19" t="n">
+        <v>4</v>
       </c>
       <c r="C25" s="20" t="inlineStr">
         <is>
@@ -2914,6 +2976,11 @@
           <t>Section E: Category Management   |   Total Marks: 8</t>
         </is>
       </c>
+      <c r="B27" s="25" t="n"/>
+      <c r="C27" s="25" t="n"/>
+      <c r="D27" s="25" t="n"/>
+      <c r="E27" s="25" t="n"/>
+      <c r="F27" s="26" t="n"/>
     </row>
     <row r="28" ht="60" customHeight="1">
       <c r="A28" s="18" t="inlineStr">
@@ -2980,10 +3047,8 @@
           <t>Demo Management (N/A)</t>
         </is>
       </c>
-      <c r="B30" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B30" s="19" t="n">
+        <v>4</v>
       </c>
       <c r="C30" s="20" t="inlineStr">
         <is>
@@ -3081,6 +3146,11 @@
           <t>Section A: Floor Management Audit   |   Total Marks: 46</t>
         </is>
       </c>
+      <c r="B3" s="25" t="n"/>
+      <c r="C3" s="25" t="n"/>
+      <c r="D3" s="25" t="n"/>
+      <c r="E3" s="25" t="n"/>
+      <c r="F3" s="26" t="n"/>
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
@@ -3299,10 +3369,8 @@
           <t>Mannequin Displays, Hot Spots, Focal Point &amp; High Point (N/A)</t>
         </is>
       </c>
-      <c r="B11" s="23" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B11" s="23" t="n">
+        <v>4</v>
       </c>
       <c r="C11" s="24" t="inlineStr">
         <is>
@@ -3391,6 +3459,11 @@
           <t>Section B: Pricing   |   Total Marks: 6</t>
         </is>
       </c>
+      <c r="B14" s="25" t="n"/>
+      <c r="C14" s="25" t="n"/>
+      <c r="D14" s="25" t="n"/>
+      <c r="E14" s="25" t="n"/>
+      <c r="F14" s="26" t="n"/>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
@@ -3452,10 +3525,8 @@
           <t>Live More Day / Buying Cycle Price Change Implementation (N/A)</t>
         </is>
       </c>
-      <c r="B17" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B17" s="19" t="n">
+        <v>4</v>
       </c>
       <c r="C17" s="20" t="inlineStr">
         <is>
@@ -3508,6 +3579,11 @@
           <t>Section C: People Management Audit   |   Total Marks: 20</t>
         </is>
       </c>
+      <c r="B19" s="25" t="n"/>
+      <c r="C19" s="25" t="n"/>
+      <c r="D19" s="25" t="n"/>
+      <c r="E19" s="25" t="n"/>
+      <c r="F19" s="26" t="n"/>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="18" t="inlineStr">
@@ -3661,6 +3737,11 @@
           <t>Section D: Merchandize Management Audit   |   Total Marks: 22</t>
         </is>
       </c>
+      <c r="B25" s="25" t="n"/>
+      <c r="C25" s="25" t="n"/>
+      <c r="D25" s="25" t="n"/>
+      <c r="E25" s="25" t="n"/>
+      <c r="F25" s="26" t="n"/>
     </row>
     <row r="26" ht="60" customHeight="1">
       <c r="A26" s="18" t="inlineStr">
@@ -3916,6 +3997,11 @@
           <t>Section A: Back End Management   |   Total Marks: 14</t>
         </is>
       </c>
+      <c r="B3" s="25" t="n"/>
+      <c r="C3" s="25" t="n"/>
+      <c r="D3" s="25" t="n"/>
+      <c r="E3" s="25" t="n"/>
+      <c r="F3" s="26" t="n"/>
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
@@ -3983,10 +4069,8 @@
           <t>Parking Management - Mall / Stand-alone Store (N/A)</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B6" s="19" t="n">
+        <v>4</v>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
@@ -4133,10 +4217,8 @@
           <t>External Warehouse / Remote (N/A)</t>
         </is>
       </c>
-      <c r="B11" s="23" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B11" s="23" t="n">
+        <v>4</v>
       </c>
       <c r="C11" s="24" t="inlineStr">
         <is>
@@ -4192,6 +4274,11 @@
           <t>Section B: Safety Management   |   Total Marks: 16</t>
         </is>
       </c>
+      <c r="B13" s="25" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="26" t="n"/>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
@@ -4432,6 +4519,11 @@
           <t>Section C: Housekeeping Management   |   Total Marks: 12</t>
         </is>
       </c>
+      <c r="B22" s="25" t="n"/>
+      <c r="C22" s="25" t="n"/>
+      <c r="D22" s="25" t="n"/>
+      <c r="E22" s="25" t="n"/>
+      <c r="F22" s="26" t="n"/>
     </row>
     <row r="23" ht="60" customHeight="1">
       <c r="A23" s="18" t="inlineStr">
@@ -4613,6 +4705,11 @@
           <t>Section D: Security &amp; Shrinkage   |   Total Marks: 26</t>
         </is>
       </c>
+      <c r="B29" s="25" t="n"/>
+      <c r="C29" s="25" t="n"/>
+      <c r="D29" s="25" t="n"/>
+      <c r="E29" s="25" t="n"/>
+      <c r="F29" s="26" t="n"/>
     </row>
     <row r="30" ht="60" customHeight="1">
       <c r="A30" s="18" t="inlineStr">
@@ -5001,6 +5098,11 @@
           <t>Section E: Maintenance Management   |   Total Marks: 10</t>
         </is>
       </c>
+      <c r="B43" s="25" t="n"/>
+      <c r="C43" s="25" t="n"/>
+      <c r="D43" s="25" t="n"/>
+      <c r="E43" s="25" t="n"/>
+      <c r="F43" s="26" t="n"/>
     </row>
     <row r="44" ht="60" customHeight="1">
       <c r="A44" s="18" t="inlineStr">
@@ -5152,6 +5254,11 @@
           <t>Section F: People Management   |   Total Marks: 5</t>
         </is>
       </c>
+      <c r="B49" s="25" t="n"/>
+      <c r="C49" s="25" t="n"/>
+      <c r="D49" s="25" t="n"/>
+      <c r="E49" s="25" t="n"/>
+      <c r="F49" s="26" t="n"/>
     </row>
     <row r="50" ht="60" customHeight="1">
       <c r="A50" s="18" t="inlineStr">
@@ -5245,6 +5352,11 @@
           <t>Section G: Store Ambience and Customer Experience   |   Total Marks: 13</t>
         </is>
       </c>
+      <c r="B53" s="25" t="n"/>
+      <c r="C53" s="25" t="n"/>
+      <c r="D53" s="25" t="n"/>
+      <c r="E53" s="25" t="n"/>
+      <c r="F53" s="26" t="n"/>
     </row>
     <row r="54" ht="60" customHeight="1">
       <c r="A54" s="18" t="inlineStr">

</xml_diff>